<commit_message>
Complete Assignment 05: Multi-agent system, benchmark evaluation matrix (350 runs), and SUBMISSION_05.md report
</commit_message>
<xml_diff>
--- a/lesson4/assignment_04.xlsx
+++ b/lesson4/assignment_04.xlsx
@@ -878,10 +878,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;amp;#xFF2D;&amp;amp;#xFF33; &amp;amp;#xFF30;&amp;amp;#x30B4;&amp;amp;#x30B7;&amp;amp;#x30C3;&amp;amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;amp;#xB9D1;&amp;amp;#xC740; &amp;amp;#xACE0;&amp;amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;amp;#x5B8B;&amp;amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;amp;#x65B0;&amp;amp;#x7D30;&amp;amp;#x660E;&amp;amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="&amp;amp;amp;#xFF2D;&amp;amp;amp;#xFF33; &amp;amp;amp;#xFF30;&amp;amp;amp;#x30B4;&amp;amp;amp;#x30B7;&amp;amp;amp;#x30C3;&amp;amp;amp;#x30AF;"/>
+        <a:font script="Hang" typeface="&amp;amp;amp;#xB9D1;&amp;amp;amp;#xC740; &amp;amp;amp;#xACE0;&amp;amp;amp;#xB515;"/>
+        <a:font script="Hans" typeface="&amp;amp;amp;#x5B8B;&amp;amp;amp;#x4F53;"/>
+        <a:font script="Hant" typeface="&amp;amp;amp;#x65B0;&amp;amp;amp;#x7D30;&amp;amp;amp;#x660E;&amp;amp;amp;#x9AD4;"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -912,10 +912,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;amp;#xFF2D;&amp;amp;#xFF33; &amp;amp;#xFF30;&amp;amp;#x30B4;&amp;amp;#x30B7;&amp;amp;#x30C3;&amp;amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;amp;#xB9D1;&amp;amp;#xC740; &amp;amp;#xACE0;&amp;amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;amp;#x5B8B;&amp;amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;amp;#x65B0;&amp;amp;#x7D30;&amp;amp;#x660E;&amp;amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="&amp;amp;amp;#xFF2D;&amp;amp;amp;#xFF33; &amp;amp;amp;#xFF30;&amp;amp;amp;#x30B4;&amp;amp;amp;#x30B7;&amp;amp;amp;#x30C3;&amp;amp;amp;#x30AF;"/>
+        <a:font script="Hang" typeface="&amp;amp;amp;#xB9D1;&amp;amp;amp;#xC740; &amp;amp;amp;#xACE0;&amp;amp;amp;#xB515;"/>
+        <a:font script="Hans" typeface="&amp;amp;amp;#x5B8B;&amp;amp;amp;#x4F53;"/>
+        <a:font script="Hant" typeface="&amp;amp;amp;#x65B0;&amp;amp;amp;#x7D30;&amp;amp;amp;#x660E;&amp;amp;amp;#x9AD4;"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1116,7 +1116,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{9E26899B-41BA-4C35-84F7-6C8761D639D2}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{40437C4A-D8A5-4EBE-9FA5-721B8ABD1A05}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1742,7 +1742,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D9933C83-4F49-4F76-B63F-C1E2278E6721}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{02FE454E-6DC3-4099-BCEC-8532FB9645E8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K501"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>

</xml_diff>